<commit_message>
[Spec Kit] Implement address postal UI progress
</commit_message>
<xml_diff>
--- a/docs/test-files/by-language/en/en_workbook.xlsx
+++ b/docs/test-files/by-language/en/en_workbook.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -527,10 +527,22 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>address</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>123 Market Street, New York, NY</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>project</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Project Falcon</t>
         </is>

</xml_diff>